<commit_message>
Update land registry Excel: add parcels 38481/28,33 and new block 401053/1
38 parcels across 4 blocks, total 1,398,610 מ"ר
</commit_message>
<xml_diff>
--- a/נסחי_רישום_בן_גוריון_תצר.xlsx
+++ b/נסחי_רישום_בן_גוריון_תצר.xlsx
@@ -41,7 +41,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -70,6 +70,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF8E1"/>
         <bgColor rgb="00FFF8E1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3E5F5"/>
+        <bgColor rgb="00F3E5F5"/>
       </patternFill>
     </fill>
     <fill>
@@ -105,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -119,7 +125,10 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -487,16 +496,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1650,23 +1659,120 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>591</v>
+      </c>
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דף 180</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>2203</v>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>מפגש דרך-מסילה (מקרקעי יעוד)</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>31/12/2018</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>מס' ישן: 38481/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>401053</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>1179179</v>
+      </c>
+      <c r="D39" s="5" t="inlineStr"/>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>מדינת ישראל (51/100) + רשות הפיתוח (49/100)</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>29/10/2025</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>גוש שומה 6 חלקה 10, גוש שומה 38063 חלקות 6,9-10, ספר ב"ש 17 דפים 180,183-184</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>סה"כ</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>35 חלקות</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="n">
-        <v>216637</v>
-      </c>
-      <c r="D37" s="5" t="inlineStr"/>
-      <c r="E37" s="5" t="inlineStr"/>
-      <c r="F37" s="5" t="inlineStr"/>
-      <c r="G37" s="5" t="inlineStr"/>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>38 חלקות</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>1398610</v>
+      </c>
+      <c r="D40" s="6" t="inlineStr"/>
+      <c r="E40" s="6" t="inlineStr"/>
+      <c r="F40" s="6" t="inlineStr"/>
+      <c r="G40" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Excel: add 38126/32 and 38480/12-15
43 parcels across 4 blocks, total 1,406,891 מ"ר
</commit_message>
<xml_diff>
--- a/נסחי_רישום_בן_גוריון_תצר.xlsx
+++ b/נסחי_רישום_בן_גוריון_תצר.xlsx
@@ -496,14 +496,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
@@ -864,33 +864,37 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>38480</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>4140</v>
-      </c>
-      <c r="D12" s="3" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>מינהל מקרקעי ישראל</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>01/01/1970</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>ספר ב"ש 5 דף 44</t>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>38126</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>1957</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>מפגש דרך-מסילה (מקרקעי יעוד)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>מדינת ישראל</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>31/12/2018</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>מס' ישן: 38126/14-15,30</t>
         </is>
       </c>
     </row>
@@ -902,11 +906,11 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1998</v>
+        <v>4140</v>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr">
@@ -933,7 +937,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
@@ -964,7 +968,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
@@ -995,7 +999,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
@@ -1026,11 +1030,11 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>4140</v>
+        <v>1998</v>
       </c>
       <c r="D17" s="3" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr">
@@ -1057,11 +1061,11 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>3500</v>
+        <v>4140</v>
       </c>
       <c r="D18" s="3" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr">
@@ -1088,17 +1092,13 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>2000</v>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>דרך (מקרקעי יעוד)</t>
-        </is>
-      </c>
+        <v>3500</v>
+      </c>
+      <c r="D19" s="3" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr">
         <is>
           <t>מינהל מקרקעי ישראל</t>
@@ -1123,15 +1123,15 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>שביל (מקרקעי יעוד)</t>
+          <t>דרך (מקרקעי יעוד)</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -1158,185 +1158,185 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>שביל (מקרקעי יעוד)</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>מינהל מקרקעי ישראל</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>01/01/1970</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 5 דף 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>38480</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="C21" s="3" t="n">
+      <c r="C22" s="3" t="n">
         <v>2800</v>
       </c>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>מינהל מקרקעי ישראל</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>01/01/1970</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>ספר ב"ש 5 דף 44</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>38481</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="n">
-        <v>4826</v>
-      </c>
-      <c r="D22" s="4" t="inlineStr"/>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>15/07/2014</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>38480</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>2896</v>
+      </c>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>11/08/2014</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>38481</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="n">
-        <v>11986</v>
-      </c>
-      <c r="D23" s="4" t="inlineStr"/>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>15/07/2014</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>38480</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>1141</v>
+      </c>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>11/08/2014</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>38481</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="n">
-        <v>7743</v>
-      </c>
-      <c r="D24" s="4" t="inlineStr"/>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>15/07/2014</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
-        </is>
-      </c>
-    </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>38481</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="n">
-        <v>1259</v>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>שביל (מקרקעי יעוד)</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>15/07/2014</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>38480</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>1143</v>
+      </c>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>11/08/2014</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>38481</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="n">
-        <v>10162</v>
-      </c>
-      <c r="D26" s="4" t="inlineStr"/>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>15/07/2014</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>38480</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>1144</v>
+      </c>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>11/08/2014</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -1348,11 +1348,11 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>6254</v>
+        <v>4826</v>
       </c>
       <c r="D27" s="4" t="inlineStr"/>
       <c r="E27" s="4" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1379,11 +1379,11 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>13354</v>
+        <v>11986</v>
       </c>
       <c r="D28" s="4" t="inlineStr"/>
       <c r="E28" s="4" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1410,11 +1410,11 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>13059</v>
+        <v>7743</v>
       </c>
       <c r="D29" s="4" t="inlineStr"/>
       <c r="E29" s="4" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1441,13 +1441,17 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>8490</v>
-      </c>
-      <c r="D30" s="4" t="inlineStr"/>
+        <v>1259</v>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>שביל (מקרקעי יעוד)</t>
+        </is>
+      </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1460,7 +1464,7 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1472,11 +1476,11 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>9066</v>
+        <v>10162</v>
       </c>
       <c r="D31" s="4" t="inlineStr"/>
       <c r="E31" s="4" t="inlineStr">
@@ -1491,7 +1495,7 @@
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1503,11 +1507,11 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>5072</v>
+        <v>6254</v>
       </c>
       <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr">
@@ -1522,7 +1526,7 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -1534,11 +1538,11 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>10986</v>
+        <v>13354</v>
       </c>
       <c r="D33" s="4" t="inlineStr"/>
       <c r="E33" s="4" t="inlineStr">
@@ -1565,11 +1569,11 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>13046</v>
+        <v>13059</v>
       </c>
       <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="inlineStr">
@@ -1596,17 +1600,13 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>482</v>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>שביל (מקרקעי יעוד)</t>
-        </is>
-      </c>
+        <v>8490</v>
+      </c>
+      <c r="D35" s="4" t="inlineStr"/>
       <c r="E35" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1619,7 +1619,7 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -1631,17 +1631,13 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>151</v>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>שביל (מקרקעי יעוד)</t>
-        </is>
-      </c>
+        <v>9066</v>
+      </c>
+      <c r="D36" s="4" t="inlineStr"/>
       <c r="E36" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1654,7 +1650,7 @@
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -1666,11 +1662,11 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>591</v>
+        <v>5072</v>
       </c>
       <c r="D37" s="4" t="inlineStr"/>
       <c r="E37" s="4" t="inlineStr">
@@ -1685,7 +1681,7 @@
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דף 180</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1697,82 +1693,245 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>10986</v>
+      </c>
+      <c r="D38" s="4" t="inlineStr"/>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>13046</v>
+      </c>
+      <c r="D39" s="4" t="inlineStr"/>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>482</v>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>שביל (מקרקעי יעוד)</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דפים 180,183</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="n">
+        <v>151</v>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>שביל (מקרקעי יעוד)</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>591</v>
+      </c>
+      <c r="D42" s="4" t="inlineStr"/>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דף 180</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
           <t>33</t>
         </is>
       </c>
-      <c r="C38" s="4" t="n">
+      <c r="C43" s="4" t="n">
         <v>2203</v>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D43" s="4" t="inlineStr">
         <is>
           <t>מפגש דרך-מסילה (מקרקעי יעוד)</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
         <is>
           <t>31/12/2018</t>
         </is>
       </c>
-      <c r="G38" s="4" t="inlineStr">
+      <c r="G43" s="4" t="inlineStr">
         <is>
           <t>מס' ישן: 38481/16</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>401053</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C39" s="5" t="n">
+      <c r="C44" s="5" t="n">
         <v>1179179</v>
       </c>
-      <c r="D39" s="5" t="inlineStr"/>
-      <c r="E39" s="5" t="inlineStr">
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t>מדינת ישראל (51/100) + רשות הפיתוח (49/100)</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr">
+      <c r="F44" s="5" t="inlineStr">
         <is>
           <t>29/10/2025</t>
         </is>
       </c>
-      <c r="G39" s="5" t="inlineStr">
+      <c r="G44" s="5" t="inlineStr">
         <is>
           <t>גוש שומה 6 חלקה 10, גוש שומה 38063 חלקות 6,9-10, ספר ב"ש 17 דפים 180,183-184</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>סה"כ</t>
         </is>
       </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>38 חלקות</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="n">
-        <v>1398610</v>
-      </c>
-      <c r="D40" s="6" t="inlineStr"/>
-      <c r="E40" s="6" t="inlineStr"/>
-      <c r="F40" s="6" t="inlineStr"/>
-      <c r="G40" s="6" t="inlineStr"/>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>43 חלקות</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>1406891</v>
+      </c>
+      <c r="D45" s="6" t="inlineStr"/>
+      <c r="E45" s="6" t="inlineStr"/>
+      <c r="F45" s="6" t="inlineStr"/>
+      <c r="G45" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Excel: add 38480/16-18 and 38481/1-2
48 parcels, total 1,445,576 מ"ר
</commit_message>
<xml_diff>
--- a/נסחי_רישום_בן_גוריון_תצר.xlsx
+++ b/נסחי_רישום_בן_גוריון_תצר.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1341,97 +1341,93 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>38481</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="n">
-        <v>4826</v>
-      </c>
-      <c r="D27" s="4" t="inlineStr"/>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>15/07/2014</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>38480</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>1146</v>
+      </c>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>11/08/2014</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>38480</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>13393</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>11/08/2014</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>38481</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="n">
-        <v>11986</v>
-      </c>
-      <c r="D28" s="4" t="inlineStr"/>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>15/07/2014</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
-        </is>
-      </c>
-    </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>38481</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="n">
-        <v>7743</v>
-      </c>
-      <c r="D29" s="4" t="inlineStr"/>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>15/07/2014</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
-        </is>
-      </c>
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>38480</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>771</v>
+      </c>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>11/08/2014</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1441,17 +1437,13 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>1259</v>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>שביל (מקרקעי יעוד)</t>
-        </is>
-      </c>
+        <v>16303</v>
+      </c>
+      <c r="D30" s="4" t="inlineStr"/>
       <c r="E30" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1476,11 +1468,11 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>10162</v>
+        <v>7072</v>
       </c>
       <c r="D31" s="4" t="inlineStr"/>
       <c r="E31" s="4" t="inlineStr">
@@ -1507,11 +1499,11 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>6254</v>
+        <v>4826</v>
       </c>
       <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr">
@@ -1526,7 +1518,7 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1538,11 +1530,11 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>13354</v>
+        <v>11986</v>
       </c>
       <c r="D33" s="4" t="inlineStr"/>
       <c r="E33" s="4" t="inlineStr">
@@ -1557,7 +1549,7 @@
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1569,11 +1561,11 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>13059</v>
+        <v>7743</v>
       </c>
       <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="inlineStr">
@@ -1588,7 +1580,7 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1600,13 +1592,17 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>8490</v>
-      </c>
-      <c r="D35" s="4" t="inlineStr"/>
+        <v>1259</v>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>שביל (מקרקעי יעוד)</t>
+        </is>
+      </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1619,7 +1615,7 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1631,11 +1627,11 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>9066</v>
+        <v>10162</v>
       </c>
       <c r="D36" s="4" t="inlineStr"/>
       <c r="E36" s="4" t="inlineStr">
@@ -1650,7 +1646,7 @@
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1662,11 +1658,11 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>5072</v>
+        <v>6254</v>
       </c>
       <c r="D37" s="4" t="inlineStr"/>
       <c r="E37" s="4" t="inlineStr">
@@ -1681,7 +1677,7 @@
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -1693,11 +1689,11 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>10986</v>
+        <v>13354</v>
       </c>
       <c r="D38" s="4" t="inlineStr"/>
       <c r="E38" s="4" t="inlineStr">
@@ -1724,11 +1720,11 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>13046</v>
+        <v>13059</v>
       </c>
       <c r="D39" s="4" t="inlineStr"/>
       <c r="E39" s="4" t="inlineStr">
@@ -1755,17 +1751,13 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>482</v>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>שביל (מקרקעי יעוד)</t>
-        </is>
-      </c>
+        <v>8490</v>
+      </c>
+      <c r="D40" s="4" t="inlineStr"/>
       <c r="E40" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1778,7 +1770,7 @@
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -1790,17 +1782,13 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>151</v>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>שביל (מקרקעי יעוד)</t>
-        </is>
-      </c>
+        <v>9066</v>
+      </c>
+      <c r="D41" s="4" t="inlineStr"/>
       <c r="E41" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1813,7 +1801,7 @@
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -1825,11 +1813,11 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>591</v>
+        <v>5072</v>
       </c>
       <c r="D42" s="4" t="inlineStr"/>
       <c r="E42" s="4" t="inlineStr">
@@ -1844,7 +1832,7 @@
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דף 180</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1856,82 +1844,245 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>10986</v>
+      </c>
+      <c r="D43" s="4" t="inlineStr"/>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="n">
+        <v>13046</v>
+      </c>
+      <c r="D44" s="4" t="inlineStr"/>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="n">
+        <v>482</v>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>שביל (מקרקעי יעוד)</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דפים 180,183</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="n">
+        <v>151</v>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>שביל (מקרקעי יעוד)</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="n">
+        <v>591</v>
+      </c>
+      <c r="D47" s="4" t="inlineStr"/>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דף 180</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
           <t>33</t>
         </is>
       </c>
-      <c r="C43" s="4" t="n">
+      <c r="C48" s="4" t="n">
         <v>2203</v>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D48" s="4" t="inlineStr">
         <is>
           <t>מפגש דרך-מסילה (מקרקעי יעוד)</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
         <is>
           <t>31/12/2018</t>
         </is>
       </c>
-      <c r="G43" s="4" t="inlineStr">
+      <c r="G48" s="4" t="inlineStr">
         <is>
           <t>מס' ישן: 38481/16</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>401053</t>
         </is>
       </c>
-      <c r="B44" s="5" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C44" s="5" t="n">
+      <c r="C49" s="5" t="n">
         <v>1179179</v>
       </c>
-      <c r="D44" s="5" t="inlineStr"/>
-      <c r="E44" s="5" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr"/>
+      <c r="E49" s="5" t="inlineStr">
         <is>
           <t>מדינת ישראל (51/100) + רשות הפיתוח (49/100)</t>
         </is>
       </c>
-      <c r="F44" s="5" t="inlineStr">
+      <c r="F49" s="5" t="inlineStr">
         <is>
           <t>29/10/2025</t>
         </is>
       </c>
-      <c r="G44" s="5" t="inlineStr">
+      <c r="G49" s="5" t="inlineStr">
         <is>
           <t>גוש שומה 6 חלקה 10, גוש שומה 38063 חלקות 6,9-10, ספר ב"ש 17 דפים 180,183-184</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="6" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>סה"כ</t>
         </is>
       </c>
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>43 חלקות</t>
-        </is>
-      </c>
-      <c r="C45" s="6" t="n">
-        <v>1406891</v>
-      </c>
-      <c r="D45" s="6" t="inlineStr"/>
-      <c r="E45" s="6" t="inlineStr"/>
-      <c r="F45" s="6" t="inlineStr"/>
-      <c r="G45" s="6" t="inlineStr"/>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>48 חלקות</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="n">
+        <v>1445576</v>
+      </c>
+      <c r="D50" s="6" t="inlineStr"/>
+      <c r="E50" s="6" t="inlineStr"/>
+      <c r="F50" s="6" t="inlineStr"/>
+      <c r="G50" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Excel: add 38481/3-7
53 parcels, total 1,459,483 מ"ר
</commit_message>
<xml_diff>
--- a/נסחי_רישום_בן_גוריון_תצר.xlsx
+++ b/נסחי_רישום_בן_גוריון_תצר.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1499,11 +1499,11 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>4826</v>
+        <v>2620</v>
       </c>
       <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr">
@@ -1530,11 +1530,11 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>11986</v>
+        <v>3473</v>
       </c>
       <c r="D33" s="4" t="inlineStr"/>
       <c r="E33" s="4" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 17 דף 180</t>
         </is>
       </c>
     </row>
@@ -1561,11 +1561,11 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>7743</v>
+        <v>2202</v>
       </c>
       <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -1592,17 +1592,13 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1259</v>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>שביל (מקרקעי יעוד)</t>
-        </is>
-      </c>
+        <v>2197</v>
+      </c>
+      <c r="D35" s="4" t="inlineStr"/>
       <c r="E35" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1615,7 +1611,7 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 8 דף 68</t>
         </is>
       </c>
     </row>
@@ -1627,11 +1623,11 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>10162</v>
+        <v>3415</v>
       </c>
       <c r="D36" s="4" t="inlineStr"/>
       <c r="E36" s="4" t="inlineStr">
@@ -1646,7 +1642,7 @@
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 8 דף 68</t>
         </is>
       </c>
     </row>
@@ -1658,11 +1654,11 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>6254</v>
+        <v>4826</v>
       </c>
       <c r="D37" s="4" t="inlineStr"/>
       <c r="E37" s="4" t="inlineStr">
@@ -1677,7 +1673,7 @@
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1689,11 +1685,11 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>13354</v>
+        <v>11986</v>
       </c>
       <c r="D38" s="4" t="inlineStr"/>
       <c r="E38" s="4" t="inlineStr">
@@ -1708,7 +1704,7 @@
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1720,11 +1716,11 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>13059</v>
+        <v>7743</v>
       </c>
       <c r="D39" s="4" t="inlineStr"/>
       <c r="E39" s="4" t="inlineStr">
@@ -1739,7 +1735,7 @@
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1751,13 +1747,17 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>8490</v>
-      </c>
-      <c r="D40" s="4" t="inlineStr"/>
+        <v>1259</v>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>שביל (מקרקעי יעוד)</t>
+        </is>
+      </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1770,7 +1770,7 @@
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1782,11 +1782,11 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>9066</v>
+        <v>10162</v>
       </c>
       <c r="D41" s="4" t="inlineStr"/>
       <c r="E41" s="4" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1813,11 +1813,11 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>5072</v>
+        <v>6254</v>
       </c>
       <c r="D42" s="4" t="inlineStr"/>
       <c r="E42" s="4" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -1844,11 +1844,11 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>10986</v>
+        <v>13354</v>
       </c>
       <c r="D43" s="4" t="inlineStr"/>
       <c r="E43" s="4" t="inlineStr">
@@ -1875,11 +1875,11 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>13046</v>
+        <v>13059</v>
       </c>
       <c r="D44" s="4" t="inlineStr"/>
       <c r="E44" s="4" t="inlineStr">
@@ -1906,17 +1906,13 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>482</v>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>שביל (מקרקעי יעוד)</t>
-        </is>
-      </c>
+        <v>8490</v>
+      </c>
+      <c r="D45" s="4" t="inlineStr"/>
       <c r="E45" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1929,7 +1925,7 @@
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -1941,17 +1937,13 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>151</v>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>שביל (מקרקעי יעוד)</t>
-        </is>
-      </c>
+        <v>9066</v>
+      </c>
+      <c r="D46" s="4" t="inlineStr"/>
       <c r="E46" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1964,7 +1956,7 @@
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -1976,11 +1968,11 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>591</v>
+        <v>5072</v>
       </c>
       <c r="D47" s="4" t="inlineStr"/>
       <c r="E47" s="4" t="inlineStr">
@@ -1995,7 +1987,7 @@
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דף 180</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -2007,82 +1999,245 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="n">
+        <v>10986</v>
+      </c>
+      <c r="D48" s="4" t="inlineStr"/>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="n">
+        <v>13046</v>
+      </c>
+      <c r="D49" s="4" t="inlineStr"/>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="n">
+        <v>482</v>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>שביל (מקרקעי יעוד)</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דפים 180,183</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="n">
+        <v>151</v>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>שביל (מקרקעי יעוד)</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="n">
+        <v>591</v>
+      </c>
+      <c r="D52" s="4" t="inlineStr"/>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דף 180</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
           <t>33</t>
         </is>
       </c>
-      <c r="C48" s="4" t="n">
+      <c r="C53" s="4" t="n">
         <v>2203</v>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D53" s="4" t="inlineStr">
         <is>
           <t>מפגש דרך-מסילה (מקרקעי יעוד)</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
         <is>
           <t>31/12/2018</t>
         </is>
       </c>
-      <c r="G48" s="4" t="inlineStr">
+      <c r="G53" s="4" t="inlineStr">
         <is>
           <t>מס' ישן: 38481/16</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>401053</t>
         </is>
       </c>
-      <c r="B49" s="5" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C49" s="5" t="n">
+      <c r="C54" s="5" t="n">
         <v>1179179</v>
       </c>
-      <c r="D49" s="5" t="inlineStr"/>
-      <c r="E49" s="5" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr"/>
+      <c r="E54" s="5" t="inlineStr">
         <is>
           <t>מדינת ישראל (51/100) + רשות הפיתוח (49/100)</t>
         </is>
       </c>
-      <c r="F49" s="5" t="inlineStr">
+      <c r="F54" s="5" t="inlineStr">
         <is>
           <t>29/10/2025</t>
         </is>
       </c>
-      <c r="G49" s="5" t="inlineStr">
+      <c r="G54" s="5" t="inlineStr">
         <is>
           <t>גוש שומה 6 חלקה 10, גוש שומה 38063 חלקות 6,9-10, ספר ב"ש 17 דפים 180,183-184</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="6" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>סה"כ</t>
         </is>
       </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>48 חלקות</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="n">
-        <v>1445576</v>
-      </c>
-      <c r="D50" s="6" t="inlineStr"/>
-      <c r="E50" s="6" t="inlineStr"/>
-      <c r="F50" s="6" t="inlineStr"/>
-      <c r="G50" s="6" t="inlineStr"/>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>53 חלקות</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="n">
+        <v>1459483</v>
+      </c>
+      <c r="D55" s="6" t="inlineStr"/>
+      <c r="E55" s="6" t="inlineStr"/>
+      <c r="F55" s="6" t="inlineStr"/>
+      <c r="G55" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Complete land registry Excel: add 38481/15,17 - all LOTLIST parcels covered
55 parcels across 4 blocks (38126, 38480, 38481, 401053), total 1,462,563 מ"ר
</commit_message>
<xml_diff>
--- a/נסחי_רישום_בן_גוריון_תצר.xlsx
+++ b/נסחי_רישום_בן_גוריון_תצר.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1813,13 +1813,17 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>6254</v>
-      </c>
-      <c r="D42" s="4" t="inlineStr"/>
+        <v>2407</v>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>דרך (מקרקעי יעוד)</t>
+        </is>
+      </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1832,7 +1836,7 @@
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1844,11 +1848,11 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>13354</v>
+        <v>673</v>
       </c>
       <c r="D43" s="4" t="inlineStr"/>
       <c r="E43" s="4" t="inlineStr">
@@ -1863,7 +1867,7 @@
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דף 180</t>
         </is>
       </c>
     </row>
@@ -1875,11 +1879,11 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>13059</v>
+        <v>6254</v>
       </c>
       <c r="D44" s="4" t="inlineStr"/>
       <c r="E44" s="4" t="inlineStr">
@@ -1906,11 +1910,11 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>8490</v>
+        <v>13354</v>
       </c>
       <c r="D45" s="4" t="inlineStr"/>
       <c r="E45" s="4" t="inlineStr">
@@ -1937,11 +1941,11 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>9066</v>
+        <v>13059</v>
       </c>
       <c r="D46" s="4" t="inlineStr"/>
       <c r="E46" s="4" t="inlineStr">
@@ -1968,11 +1972,11 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>5072</v>
+        <v>8490</v>
       </c>
       <c r="D47" s="4" t="inlineStr"/>
       <c r="E47" s="4" t="inlineStr">
@@ -1987,7 +1991,7 @@
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -1999,11 +2003,11 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>10986</v>
+        <v>9066</v>
       </c>
       <c r="D48" s="4" t="inlineStr"/>
       <c r="E48" s="4" t="inlineStr">
@@ -2030,11 +2034,11 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>13046</v>
+        <v>5072</v>
       </c>
       <c r="D49" s="4" t="inlineStr"/>
       <c r="E49" s="4" t="inlineStr">
@@ -2049,7 +2053,7 @@
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -2061,17 +2065,13 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>482</v>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>שביל (מקרקעי יעוד)</t>
-        </is>
-      </c>
+        <v>10986</v>
+      </c>
+      <c r="D50" s="4" t="inlineStr"/>
       <c r="E50" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -2084,7 +2084,7 @@
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -2096,17 +2096,13 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>25</t>
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>151</v>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>שביל (מקרקעי יעוד)</t>
-        </is>
-      </c>
+        <v>13046</v>
+      </c>
+      <c r="D51" s="4" t="inlineStr"/>
       <c r="E51" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -2119,7 +2115,7 @@
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -2131,13 +2127,17 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>26</t>
         </is>
       </c>
       <c r="C52" s="4" t="n">
-        <v>591</v>
-      </c>
-      <c r="D52" s="4" t="inlineStr"/>
+        <v>482</v>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>שביל (מקרקעי יעוד)</t>
+        </is>
+      </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -2150,7 +2150,7 @@
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דף 180</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -2162,82 +2162,148 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="n">
+        <v>151</v>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>שביל (מקרקעי יעוד)</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="n">
+        <v>591</v>
+      </c>
+      <c r="D54" s="4" t="inlineStr"/>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דף 180</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
           <t>33</t>
         </is>
       </c>
-      <c r="C53" s="4" t="n">
+      <c r="C55" s="4" t="n">
         <v>2203</v>
       </c>
-      <c r="D53" s="4" t="inlineStr">
+      <c r="D55" s="4" t="inlineStr">
         <is>
           <t>מפגש דרך-מסילה (מקרקעי יעוד)</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
         <is>
           <t>31/12/2018</t>
         </is>
       </c>
-      <c r="G53" s="4" t="inlineStr">
+      <c r="G55" s="4" t="inlineStr">
         <is>
           <t>מס' ישן: 38481/16</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>401053</t>
         </is>
       </c>
-      <c r="B54" s="5" t="inlineStr">
+      <c r="B56" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C54" s="5" t="n">
+      <c r="C56" s="5" t="n">
         <v>1179179</v>
       </c>
-      <c r="D54" s="5" t="inlineStr"/>
-      <c r="E54" s="5" t="inlineStr">
+      <c r="D56" s="5" t="inlineStr"/>
+      <c r="E56" s="5" t="inlineStr">
         <is>
           <t>מדינת ישראל (51/100) + רשות הפיתוח (49/100)</t>
         </is>
       </c>
-      <c r="F54" s="5" t="inlineStr">
+      <c r="F56" s="5" t="inlineStr">
         <is>
           <t>29/10/2025</t>
         </is>
       </c>
-      <c r="G54" s="5" t="inlineStr">
+      <c r="G56" s="5" t="inlineStr">
         <is>
           <t>גוש שומה 6 חלקה 10, גוש שומה 38063 חלקות 6,9-10, ספר ב"ש 17 דפים 180,183-184</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
         <is>
           <t>סה"כ</t>
         </is>
       </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>53 חלקות</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="n">
-        <v>1459483</v>
-      </c>
-      <c r="D55" s="6" t="inlineStr"/>
-      <c r="E55" s="6" t="inlineStr"/>
-      <c r="F55" s="6" t="inlineStr"/>
-      <c r="G55" s="6" t="inlineStr"/>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>55 חלקות</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="n">
+        <v>1462563</v>
+      </c>
+      <c r="D57" s="6" t="inlineStr"/>
+      <c r="E57" s="6" t="inlineStr"/>
+      <c r="F57" s="6" t="inlineStr"/>
+      <c r="G57" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Final Excel: 43 verified parcels from actual PDFs
All parcels match LOTLIST, total 1,423,038 מ"ר
</commit_message>
<xml_diff>
--- a/נסחי_רישום_בן_גוריון_תצר.xlsx
+++ b/נסחי_רישום_בן_גוריון_תצר.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -588,11 +588,11 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2896</v>
+        <v>3103</v>
       </c>
       <c r="D3" s="3" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr">
@@ -619,11 +619,11 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1141</v>
+        <v>2195</v>
       </c>
       <c r="D4" s="3" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -650,11 +650,11 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1143</v>
+        <v>2196</v>
       </c>
       <c r="D5" s="3" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr">
@@ -681,11 +681,11 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>1144</v>
+        <v>2199</v>
       </c>
       <c r="D6" s="3" t="inlineStr"/>
       <c r="E6" s="3" t="inlineStr">
@@ -712,11 +712,11 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>1146</v>
+        <v>2202</v>
       </c>
       <c r="D7" s="3" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr">
@@ -743,11 +743,11 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>13393</v>
+        <v>2203</v>
       </c>
       <c r="D8" s="3" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -774,272 +774,280 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>7924</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>דרך (מקרקעי יעוד)</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>11/08/2014</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דפים 180,183</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>38480</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>39154</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>מסילת ברזל (מקרקעי יעוד)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>11/08/2014</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>38480</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>2896</v>
+      </c>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>11/08/2014</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דפים 180,183</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>38480</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>1141</v>
+      </c>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>11/08/2014</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דפים 180,183</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>38480</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>1143</v>
+      </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>11/08/2014</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דף 183</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>38480</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>1144</v>
+      </c>
+      <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>11/08/2014</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>38480</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>1146</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>11/08/2014</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>38480</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>13393</v>
+      </c>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>11/08/2014</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דפים 180,183</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>38480</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
           <t>18</t>
         </is>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C17" s="3" t="n">
         <v>771</v>
       </c>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>11/08/2014</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>38481</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>16303</v>
-      </c>
-      <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>15/07/2014</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>38481</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>7072</v>
-      </c>
-      <c r="D11" s="4" t="inlineStr"/>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>15/07/2014</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>38481</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>2620</v>
-      </c>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>15/07/2014</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>38481</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="n">
-        <v>3473</v>
-      </c>
-      <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>15/07/2014</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>ספר ב"ש 17 דף 180</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>38481</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>2202</v>
-      </c>
-      <c r="D14" s="4" t="inlineStr"/>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>15/07/2014</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>38481</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="n">
-        <v>2197</v>
-      </c>
-      <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>15/07/2014</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>ספר ב"ש 8 דף 68</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>38481</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>3415</v>
-      </c>
-      <c r="D16" s="4" t="inlineStr"/>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>15/07/2014</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>ספר ב"ש 8 דף 68</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>38481</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="n">
-        <v>4826</v>
-      </c>
-      <c r="D17" s="4" t="inlineStr"/>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>15/07/2014</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
-        </is>
-      </c>
+      <c r="G17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1049,11 +1057,11 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>11986</v>
+        <v>16303</v>
       </c>
       <c r="D18" s="4" t="inlineStr"/>
       <c r="E18" s="4" t="inlineStr">
@@ -1080,11 +1088,11 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>7743</v>
+        <v>7072</v>
       </c>
       <c r="D19" s="4" t="inlineStr"/>
       <c r="E19" s="4" t="inlineStr">
@@ -1111,17 +1119,13 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>1259</v>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>שביל (מקרקעי יעוד)</t>
-        </is>
-      </c>
+        <v>2620</v>
+      </c>
+      <c r="D20" s="4" t="inlineStr"/>
       <c r="E20" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1146,11 +1150,11 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>10162</v>
+        <v>3473</v>
       </c>
       <c r="D21" s="4" t="inlineStr"/>
       <c r="E21" s="4" t="inlineStr">
@@ -1165,7 +1169,7 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 17 דף 180</t>
         </is>
       </c>
     </row>
@@ -1177,17 +1181,13 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>2407</v>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>דרך (מקרקעי יעוד)</t>
-        </is>
-      </c>
+        <v>2202</v>
+      </c>
+      <c r="D22" s="4" t="inlineStr"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -1212,11 +1212,11 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>673</v>
+        <v>2197</v>
       </c>
       <c r="D23" s="4" t="inlineStr"/>
       <c r="E23" s="4" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דף 180</t>
+          <t>ספר ב"ש 8 דף 68</t>
         </is>
       </c>
     </row>
@@ -1243,11 +1243,11 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>6254</v>
+        <v>3415</v>
       </c>
       <c r="D24" s="4" t="inlineStr"/>
       <c r="E24" s="4" t="inlineStr">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 8 דף 68</t>
         </is>
       </c>
     </row>
@@ -1274,11 +1274,11 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>13354</v>
+        <v>4826</v>
       </c>
       <c r="D25" s="4" t="inlineStr"/>
       <c r="E25" s="4" t="inlineStr">
@@ -1293,7 +1293,7 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1305,11 +1305,11 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>13059</v>
+        <v>11986</v>
       </c>
       <c r="D26" s="4" t="inlineStr"/>
       <c r="E26" s="4" t="inlineStr">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1336,11 +1336,11 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>8490</v>
+        <v>7743</v>
       </c>
       <c r="D27" s="4" t="inlineStr"/>
       <c r="E27" s="4" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1367,13 +1367,17 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>9066</v>
-      </c>
-      <c r="D28" s="4" t="inlineStr"/>
+        <v>1259</v>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>שביל (מקרקעי יעוד)</t>
+        </is>
+      </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1386,7 +1390,7 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1398,11 +1402,11 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>5072</v>
+        <v>10162</v>
       </c>
       <c r="D29" s="4" t="inlineStr"/>
       <c r="E29" s="4" t="inlineStr">
@@ -1429,13 +1433,17 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>10986</v>
-      </c>
-      <c r="D30" s="4" t="inlineStr"/>
+        <v>2407</v>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>דרך (מקרקעי יעוד)</t>
+        </is>
+      </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1448,7 +1456,7 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דפים 180,183</t>
         </is>
       </c>
     </row>
@@ -1460,11 +1468,11 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>13046</v>
+        <v>673</v>
       </c>
       <c r="D31" s="4" t="inlineStr"/>
       <c r="E31" s="4" t="inlineStr">
@@ -1479,7 +1487,7 @@
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+          <t>ספר ב"ש 17 דף 180</t>
         </is>
       </c>
     </row>
@@ -1491,17 +1499,13 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>482</v>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>שביל (מקרקעי יעוד)</t>
-        </is>
-      </c>
+        <v>6254</v>
+      </c>
+      <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1514,7 +1518,7 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דפים 180,183</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -1526,17 +1530,13 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>151</v>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>שביל (מקרקעי יעוד)</t>
-        </is>
-      </c>
+        <v>13354</v>
+      </c>
+      <c r="D33" s="4" t="inlineStr"/>
       <c r="E33" s="4" t="inlineStr">
         <is>
           <t>רשות הפתוח</t>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 8 דף 68</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -1561,11 +1561,11 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>591</v>
+        <v>13059</v>
       </c>
       <c r="D34" s="4" t="inlineStr"/>
       <c r="E34" s="4" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>ספר ב"ש 17 דף 180</t>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
         </is>
       </c>
     </row>
@@ -1592,82 +1592,338 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>8490</v>
+      </c>
+      <c r="D35" s="4" t="inlineStr"/>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>9066</v>
+      </c>
+      <c r="D36" s="4" t="inlineStr"/>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>5072</v>
+      </c>
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דפים 180,183</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>10986</v>
+      </c>
+      <c r="D38" s="4" t="inlineStr"/>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>13046</v>
+      </c>
+      <c r="D39" s="4" t="inlineStr"/>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68, ספר ב"ש 17 דף 183</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>482</v>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>שביל (מקרקעי יעוד)</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דפים 180,183</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="n">
+        <v>151</v>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>שביל (מקרקעי יעוד)</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 8 דף 68</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>591</v>
+      </c>
+      <c r="D42" s="4" t="inlineStr"/>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>15/07/2014</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>ספר ב"ש 17 דף 180</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>38481</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
           <t>33</t>
         </is>
       </c>
-      <c r="C35" s="4" t="n">
+      <c r="C43" s="4" t="n">
         <v>2203</v>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D43" s="4" t="inlineStr">
         <is>
           <t>מפגש דרך-מסילה (מקרקעי יעוד)</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>רשות הפתוח</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>רשות הפתוח</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
         <is>
           <t>31/12/2018</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
+      <c r="G43" s="4" t="inlineStr">
         <is>
           <t>מס' ישן: 38481/16</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>401053</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C36" s="5" t="n">
+      <c r="C44" s="5" t="n">
         <v>1179179</v>
       </c>
-      <c r="D36" s="5" t="inlineStr"/>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t>מדינת ישראל (51/100) + רשות הפיתוח (49/100)</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="F44" s="5" t="inlineStr">
         <is>
           <t>29/10/2025</t>
         </is>
       </c>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="G44" s="5" t="inlineStr">
         <is>
           <t>גוש שומה 6 חלקה 10, גוש שומה 38063 חלקות 6,9-10, ספר ב"ש 17 דפים 180,183-184</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="6" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>סה"כ</t>
         </is>
       </c>
-      <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t>35 חלקות</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="n">
-        <v>1361862</v>
-      </c>
-      <c r="D37" s="6" t="inlineStr"/>
-      <c r="E37" s="6" t="inlineStr"/>
-      <c r="F37" s="6" t="inlineStr"/>
-      <c r="G37" s="6" t="inlineStr"/>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>43 חלקות</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>1423038</v>
+      </c>
+      <c r="D45" s="6" t="inlineStr"/>
+      <c r="E45" s="6" t="inlineStr"/>
+      <c r="F45" s="6" t="inlineStr"/>
+      <c r="G45" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>